<commit_message>
fix: replace all custom colors with strict Hissa DS tokens
- #A05C45 (custom muted red) → #B42318 (DS error primary)
- #3F7D5A (custom muted green) → #027A48 (DS success-700)
- #5A8A72 (custom green) → #039855 (DS success primary)
- #1C1C1E/#2C2C2E (dark grays) → #071437 (DS heading)
- #C4C4C4 → #99A1B7 (DS muted)
- #D1D5DB → #DBDFE9 (DS field border)
- #F3F4F6 → #F1F1F4 (DS container border)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Book2.xlsx
+++ b/Book2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Admin/Work/Code/Claude_codebase_test/esop_exercise_tax_calc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC4B74E-294B-A74E-AEBA-6F31902155F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D418EB67-42B0-9045-9D58-0F013402D41B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5180" yWindow="1800" windowWidth="28040" windowHeight="17440" xr2:uid="{84E36E02-73E5-AB43-A975-AE15F6DBCF1E}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>Grant Id</t>
   </si>
@@ -69,6 +69,15 @@
   </si>
   <si>
     <t>ROUND_DOWN</t>
+  </si>
+  <si>
+    <t>G3</t>
+  </si>
+  <si>
+    <t>G4</t>
+  </si>
+  <si>
+    <t>G5</t>
   </si>
 </sst>
 </file>
@@ -76,9 +85,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -91,6 +100,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -114,10 +130,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,16 +469,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFB3DE92-82E5-D14F-8430-C400B448E474}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.6640625" customWidth="1"/>
     <col min="6" max="6" width="19.33203125" customWidth="1"/>
     <col min="7" max="7" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,7 +503,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -507,7 +526,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -521,7 +540,7 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="F3">
         <v>1</v>
@@ -529,6 +548,87 @@
       <c r="G3" t="s">
         <v>9</v>
       </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2">
+        <v>45444</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>100</v>
+      </c>
+      <c r="E4">
+        <v>50</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="O4" s="2"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2">
+        <v>45658</v>
+      </c>
+      <c r="C5">
+        <v>100</v>
+      </c>
+      <c r="D5">
+        <v>100</v>
+      </c>
+      <c r="E5">
+        <v>25</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>9</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="M5" s="2"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46082</v>
+      </c>
+      <c r="C6">
+        <v>100</v>
+      </c>
+      <c r="D6">
+        <v>100</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="M6" s="3"/>
+      <c r="O6" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>